<commit_message>
Gjort kode klar til kjørring
Primært jobbet med forutsetningsscript.
</commit_message>
<xml_diff>
--- a/Data/BaseData/id_ir_26.xlsx
+++ b/Data/BaseData/id_ir_26.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nveazure.sharepoint.com/sites/ORG-RME-OE/Delte dokumenter/Inntektsrammer/2026/Foreløpige beregninger/IRiR2026/Data/BaseData/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nveazure-my.sharepoint.com/personal/clso_nve_no/Documents/Dokumenter/GitHub/IRiR/Data/BaseData/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="77" documentId="8_{301F8B09-BA88-4129-BE9F-DB56EBA5FCDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8DBA814A-84D0-4BFE-8BA4-B9C1A6C2FF58}"/>
+  <xr:revisionPtr revIDLastSave="83" documentId="8_{301F8B09-BA88-4129-BE9F-DB56EBA5FCDB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1B99BC3E-E6EA-435D-A31C-52FDFFAD7486}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1515" yWindow="1395" windowWidth="19185" windowHeight="10065" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="id" sheetId="1" r:id="rId1"/>
@@ -840,9 +840,10 @@
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="42" applyBorder="1"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="43">
     <cellStyle name="20 % – uthevingsfarge 1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1199,15 +1200,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C139"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:E139"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="10.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="43.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.54296875" customWidth="1"/>
+    <col min="1" max="1" width="10.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="43.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.5703125" customWidth="1"/>
+    <col min="5" max="5" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1218,7 +1220,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>982974011</v>
       </c>
@@ -1229,7 +1231,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>915729290</v>
       </c>
@@ -1240,7 +1242,7 @@
         <v>753</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>925336637</v>
       </c>
@@ -1251,7 +1253,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>921680554</v>
       </c>
@@ -1262,7 +1264,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>979151950</v>
       </c>
@@ -1273,7 +1275,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>917743193</v>
       </c>
@@ -1284,7 +1286,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>971058854</v>
       </c>
@@ -1295,7 +1297,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>953181606</v>
       </c>
@@ -1306,7 +1308,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>976944801</v>
       </c>
@@ -1317,7 +1319,7 @@
         <v>566</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>924527994</v>
       </c>
@@ -1328,7 +1330,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>923934138</v>
       </c>
@@ -1339,7 +1341,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>924862602</v>
       </c>
@@ -1350,7 +1352,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>979379455</v>
       </c>
@@ -1361,7 +1363,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>986347801</v>
       </c>
@@ -1372,7 +1374,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>979497482</v>
       </c>
@@ -1383,7 +1385,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>923488960</v>
       </c>
@@ -1394,7 +1396,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>980489698</v>
       </c>
@@ -1405,7 +1407,7 @@
         <v>675</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>918312730</v>
       </c>
@@ -1416,7 +1418,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>882783022</v>
       </c>
@@ -1427,7 +1429,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>966731508</v>
       </c>
@@ -1438,7 +1440,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>915635857</v>
       </c>
@@ -1449,7 +1451,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>923354204</v>
       </c>
@@ -1460,7 +1462,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>987626844</v>
       </c>
@@ -1471,7 +1473,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>925549738</v>
       </c>
@@ -1482,7 +1484,7 @@
         <v>659</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>981915550</v>
       </c>
@@ -1493,7 +1495,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>953681781</v>
       </c>
@@ -1504,7 +1506,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>976894677</v>
       </c>
@@ -1515,7 +1517,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>971589752</v>
       </c>
@@ -1526,7 +1528,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>924004150</v>
       </c>
@@ -1537,7 +1539,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>923050612</v>
       </c>
@@ -1548,7 +1550,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>998509289</v>
       </c>
@@ -1559,7 +1561,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>917537534</v>
       </c>
@@ -1570,7 +1572,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>930187240</v>
       </c>
@@ -1581,7 +1583,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>985411131</v>
       </c>
@@ -1592,7 +1594,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>919415096</v>
       </c>
@@ -1603,7 +1605,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>914385261</v>
       </c>
@@ -1614,7 +1616,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>824914982</v>
       </c>
@@ -1625,7 +1627,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>977285712</v>
       </c>
@@ -1636,7 +1638,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>923436596</v>
       </c>
@@ -1647,7 +1649,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>923789324</v>
       </c>
@@ -1658,7 +1660,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>913680294</v>
       </c>
@@ -1669,7 +1671,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>923152601</v>
       </c>
@@ -1680,7 +1682,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>979422679</v>
       </c>
@@ -1691,7 +1693,7 @@
         <v>611</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>924868759</v>
       </c>
@@ -1702,7 +1704,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>917424799</v>
       </c>
@@ -1713,7 +1715,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>912631532</v>
       </c>
@@ -1724,7 +1726,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>980038408</v>
       </c>
@@ -1735,7 +1737,7 @@
         <v>511</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>982897327</v>
       </c>
@@ -1746,7 +1748,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>924934867</v>
       </c>
@@ -1757,7 +1759,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>923833706</v>
       </c>
@@ -1768,7 +1770,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>925668389</v>
       </c>
@@ -1779,7 +1781,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>919173122</v>
       </c>
@@ -1789,8 +1791,9 @@
       <c r="C53">
         <v>116</v>
       </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.35">
+      <c r="E53" s="2"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>917856222</v>
       </c>
@@ -1801,7 +1804,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>921025610</v>
       </c>
@@ -1812,7 +1815,7 @@
         <v>743</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>923993355</v>
       </c>
@@ -1823,7 +1826,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>921688679</v>
       </c>
@@ -1834,7 +1837,7 @@
         <v>903</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>995204517</v>
       </c>
@@ -1845,7 +1848,7 @@
         <v>901</v>
       </c>
     </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>980824586</v>
       </c>
@@ -1856,7 +1859,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>824701482</v>
       </c>
@@ -1867,7 +1870,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>980234088</v>
       </c>
@@ -1878,7 +1881,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>996732673</v>
       </c>
@@ -1889,7 +1892,7 @@
         <v>902</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>976723805</v>
       </c>
@@ -1900,7 +1903,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>968398083</v>
       </c>
@@ -1911,7 +1914,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>925017809</v>
       </c>
@@ -1922,7 +1925,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>925067911</v>
       </c>
@@ -1933,7 +1936,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>926377841</v>
       </c>
@@ -1944,7 +1947,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>919884452</v>
       </c>
@@ -1955,7 +1958,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>954090493</v>
       </c>
@@ -1966,7 +1969,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>920295975</v>
       </c>
@@ -1977,7 +1980,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>923819177</v>
       </c>
@@ -1988,7 +1991,7 @@
         <v>274</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>985294836</v>
       </c>
@@ -1999,7 +2002,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>924940379</v>
       </c>
@@ -2010,7 +2013,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>987059729</v>
       </c>
@@ -2021,7 +2024,7 @@
         <v>685</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>962986633</v>
       </c>
@@ -2032,7 +2035,7 @@
         <v>319</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>925354813</v>
       </c>
@@ -2043,7 +2046,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>922694435</v>
       </c>
@@ -2054,7 +2057,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>924330678</v>
       </c>
@@ -2065,7 +2068,7 @@
         <v>599</v>
       </c>
     </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>924619260</v>
       </c>
@@ -2076,7 +2079,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>997712099</v>
       </c>
@@ -2087,7 +2090,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>916574894</v>
       </c>
@@ -2098,7 +2101,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>988807648</v>
       </c>
@@ -2109,7 +2112,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>978631029</v>
       </c>
@@ -2120,7 +2123,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>925315958</v>
       </c>
@@ -2131,7 +2134,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>916763476</v>
       </c>
@@ -2142,7 +2145,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>917983550</v>
       </c>
@@ -2153,7 +2156,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>965809090</v>
       </c>
@@ -2164,7 +2167,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>971040246</v>
       </c>
@@ -2175,7 +2178,7 @@
         <v>287</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>967670170</v>
       </c>
@@ -2186,7 +2189,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>824368082</v>
       </c>
@@ -2197,7 +2200,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>968168134</v>
       </c>
@@ -2208,7 +2211,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>979399901</v>
       </c>
@@ -2219,7 +2222,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>925803375</v>
       </c>
@@ -2230,7 +2233,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>916319908</v>
       </c>
@@ -2241,7 +2244,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>921683057</v>
       </c>
@@ -2252,7 +2255,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>918999361</v>
       </c>
@@ -2263,7 +2266,7 @@
         <v>625</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>984015666</v>
       </c>
@@ -2274,7 +2277,7 @@
         <v>686</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>933584801</v>
       </c>
@@ -2285,7 +2288,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="139" spans="2:2" x14ac:dyDescent="0.35">
+    <row r="139" spans="2:2" x14ac:dyDescent="0.25">
       <c r="B139" s="1"/>
     </row>
   </sheetData>
@@ -2299,6 +2302,47 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="64152832-9f03-4628-8f8a-984f7e09cd82" ContentTypeId="0x0101" PreviousValue="false"/>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <Vedtattdato xmlns="caf9241f-7654-46e4-b38c-0683f7584438">2021-03-02T00:00:00+00:00</Vedtattdato>
+    <Prosess xmlns="caf9241f-7654-46e4-b38c-0683f7584438" xsi:nil="true"/>
+    <TaxCatchAll xmlns="08670d86-fc33-4f61-bf51-96e019343c8b" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="caf9241f-7654-46e4-b38c-0683f7584438">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <g98ade60b1a5493f9b7127fdb0eec544 xmlns="08670d86-fc33-4f61-bf51-96e019343c8b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </g98ade60b1a5493f9b7127fdb0eec544>
+    <n3e020d9d98c48dbb65f924b9bc22a2a xmlns="08670d86-fc33-4f61-bf51-96e019343c8b">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </n3e020d9d98c48dbb65f924b9bc22a2a>
+    <TaxCatchAllLabel xmlns="08670d86-fc33-4f61-bf51-96e019343c8b" xsi:nil="true"/>
+    <fb87f3f3a1014cb4ad0ec65499e03bb4 xmlns="caf9241f-7654-46e4-b38c-0683f7584438">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </fb87f3f3a1014cb4ad0ec65499e03bb4>
+    <Slette_x003f_ xmlns="caf9241f-7654-46e4-b38c-0683f7584438" xsi:nil="true"/>
+    <h5401ff79c16481cab8da1bb26f238ab xmlns="caf9241f-7654-46e4-b38c-0683f7584438">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </h5401ff79c16481cab8da1bb26f238ab>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Word-dokument" ma:contentTypeID="0x010100098B676CC530A34A9FB1F4ACAD0C0A17" ma:contentTypeVersion="35" ma:contentTypeDescription="Opprett et nytt dokument." ma:contentTypeScope="" ma:versionID="32bac50741fd7a29ba3d71556f388968">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="caf9241f-7654-46e4-b38c-0683f7584438" xmlns:ns3="08670d86-fc33-4f61-bf51-96e019343c8b" xmlns:ns4="286bd567-8383-458b-8b10-610e1dbf4dce" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="e3bdb6b18078f058c2f3788d7e990f1a" ns2:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="caf9241f-7654-46e4-b38c-0683f7584438"/>
@@ -2630,52 +2674,23 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <Vedtattdato xmlns="caf9241f-7654-46e4-b38c-0683f7584438">2021-03-02T00:00:00+00:00</Vedtattdato>
-    <Prosess xmlns="caf9241f-7654-46e4-b38c-0683f7584438" xsi:nil="true"/>
-    <TaxCatchAll xmlns="08670d86-fc33-4f61-bf51-96e019343c8b" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="caf9241f-7654-46e4-b38c-0683f7584438">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <g98ade60b1a5493f9b7127fdb0eec544 xmlns="08670d86-fc33-4f61-bf51-96e019343c8b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </g98ade60b1a5493f9b7127fdb0eec544>
-    <n3e020d9d98c48dbb65f924b9bc22a2a xmlns="08670d86-fc33-4f61-bf51-96e019343c8b">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </n3e020d9d98c48dbb65f924b9bc22a2a>
-    <TaxCatchAllLabel xmlns="08670d86-fc33-4f61-bf51-96e019343c8b" xsi:nil="true"/>
-    <fb87f3f3a1014cb4ad0ec65499e03bb4 xmlns="caf9241f-7654-46e4-b38c-0683f7584438">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </fb87f3f3a1014cb4ad0ec65499e03bb4>
-    <Slette_x003f_ xmlns="caf9241f-7654-46e4-b38c-0683f7584438" xsi:nil="true"/>
-    <h5401ff79c16481cab8da1bb26f238ab xmlns="caf9241f-7654-46e4-b38c-0683f7584438">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </h5401ff79c16481cab8da1bb26f238ab>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<SharedContentType xmlns="Microsoft.SharePoint.Taxonomy.ContentTypeSync" SourceId="64152832-9f03-4628-8f8a-984f7e09cd82" ContentTypeId="0x0101" PreviousValue="false"/>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01349B33-4082-43F5-A6CD-B3BA55396486}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7981826-1DD6-4A82-844D-73D2A0F2CA28}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3745CE7B-DF66-4995-A454-797808D64E09}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{502CDE3F-B225-46AB-A56B-33DA7E645950}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2686,18 +2701,22 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3745CE7B-DF66-4995-A454-797808D64E09}">
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{01349B33-4082-43F5-A6CD-B3BA55396486}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7981826-1DD6-4A82-844D-73D2A0F2CA28}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="Microsoft.SharePoint.Taxonomy.ContentTypeSync"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="caf9241f-7654-46e4-b38c-0683f7584438"/>
+    <ds:schemaRef ds:uri="08670d86-fc33-4f61-bf51-96e019343c8b"/>
+    <ds:schemaRef ds:uri="286bd567-8383-458b-8b10-610e1dbf4dce"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>